<commit_message>
Updated EVM Calculations Spreadsheet for Sprint 1
</commit_message>
<xml_diff>
--- a/Evidence/PP/EVM Calculations/EVM Calculations Sprint 1.xlsx
+++ b/Evidence/PP/EVM Calculations/EVM Calculations Sprint 1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neelp\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4B3FBD3-DBAC-48FD-81B8-B52A06A0087E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F6397D-E0BE-4E32-B9B0-AF6B87E4A7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{62BBB4B8-20C5-4716-8AF8-DEF5FB1D4536}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{62BBB4B8-20C5-4716-8AF8-DEF5FB1D4536}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="51">
   <si>
     <t>EVM Sprint 1</t>
   </si>
@@ -101,15 +101,9 @@
     <t xml:space="preserve">Hourly Rate </t>
   </si>
   <si>
-    <t>38*4=152</t>
-  </si>
-  <si>
     <t>Cost per Point</t>
   </si>
   <si>
-    <t>(152*15)/35=£65.14 per point</t>
-  </si>
-  <si>
     <t>GBP</t>
   </si>
   <si>
@@ -164,9 +158,6 @@
     <t>Units Contributed</t>
   </si>
   <si>
-    <t>Cost Contribution</t>
-  </si>
-  <si>
     <t>Raiyan</t>
   </si>
   <si>
@@ -192,6 +183,12 @@
   </si>
   <si>
     <t>Calculate</t>
+  </si>
+  <si>
+    <t>Cost Contribution (£60/unit)</t>
+  </si>
+  <si>
+    <t>(124*15)/35=£53.14 per point</t>
   </si>
 </sst>
 </file>
@@ -230,10 +227,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -253,6 +249,265 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>36304</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>165652</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>344693</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>23501</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{05F390E6-645B-65C9-B70D-5902CA9E82EB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8492847" y="165652"/>
+          <a:ext cx="4905237" cy="3502197"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>382242</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>36305</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>692992</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>94283</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC2E1AA7-E7EA-F726-1E6F-CE68B9592C75}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5956438" y="3680653"/>
+          <a:ext cx="6390184" cy="1333500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>224439</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>63087</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>391380</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>152262</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85C641E3-D097-CAAD-8847-F810C99E8E62}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10229830" y="4982957"/>
+          <a:ext cx="4457333" cy="4462392"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>61153</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>163719</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1343713</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>63735</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C724E2DF-1A72-0B60-2B62-50B79C9A40A9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="61153" y="6176893"/>
+          <a:ext cx="5100843" cy="3179929"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1331567</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>124239</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>716294</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>57978</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7781F530-08C8-538A-DB8B-7A4332CF9AA4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5149850" y="6137413"/>
+          <a:ext cx="4826401" cy="3031435"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -284,7 +539,9 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{BB0E2826-A6F7-4A1A-82CB-ADA34D86C350}" name="Team Member"/>
     <tableColumn id="2" xr3:uid="{745D4D8A-2FBC-47AA-9D60-5C1108E4A23F}" name="Units Contributed"/>
-    <tableColumn id="3" xr3:uid="{76268C88-B98A-4433-80B7-E77D1F221973}" name="Cost Contribution" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{76268C88-B98A-4433-80B7-E77D1F221973}" name="Cost Contribution (£60/unit)" dataDxfId="0">
+      <calculatedColumnFormula>Table3[[#This Row],[Units Contributed]]*60</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -631,30 +888,31 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="2">
-        <v>2280</v>
+        <v>26</v>
+      </c>
+      <c r="B4" s="1">
+        <f>C32</f>
+        <v>1860</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E4" t="s">
         <v>1</v>
@@ -665,13 +923,14 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B5" s="2">
-        <v>2280</v>
+        <v>27</v>
+      </c>
+      <c r="B5" s="1">
+        <f>C32</f>
+        <v>1860</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
         <v>2</v>
@@ -679,20 +938,20 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="2">
-        <v>2280</v>
+        <v>28</v>
+      </c>
+      <c r="B6" s="1">
+        <f>C32</f>
+        <v>1860</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B7" s="2"/>
       <c r="E7" t="s">
         <v>4</v>
       </c>
@@ -702,14 +961,14 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="2">
+        <v>30</v>
+      </c>
+      <c r="B8">
         <f>B4-B6</f>
         <v>0</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
         <v>5</v>
@@ -720,14 +979,14 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="2">
+        <v>29</v>
+      </c>
+      <c r="B9">
         <f>B4-B5</f>
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
         <v>6</v>
@@ -737,7 +996,6 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B10" s="2"/>
       <c r="E10" t="s">
         <v>7</v>
       </c>
@@ -747,9 +1005,9 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="2">
+        <v>31</v>
+      </c>
+      <c r="B11">
         <f>B4/B6</f>
         <v>1</v>
       </c>
@@ -760,9 +1018,9 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="2">
+        <v>32</v>
+      </c>
+      <c r="B12">
         <f>B4/B5</f>
         <v>1</v>
       </c>
@@ -774,7 +1032,6 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B13" s="2"/>
       <c r="E13" t="s">
         <v>9</v>
       </c>
@@ -784,42 +1041,43 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="2">
-        <v>2280</v>
+        <v>35</v>
+      </c>
+      <c r="B14" s="1">
+        <f>C32</f>
+        <v>1860</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B15">
         <f>B14/B11</f>
-        <v>2280</v>
+        <v>1860</v>
       </c>
       <c r="C15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B16">
         <f>B14-B15</f>
         <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19">
         <v>35</v>
@@ -829,13 +1087,14 @@
       <c r="A20" t="s">
         <v>19</v>
       </c>
-      <c r="B20" t="s">
-        <v>21</v>
+      <c r="B20">
+        <f>B32*4</f>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B21" s="1">
         <v>30000</v>
@@ -849,81 +1108,85 @@
         <v>15</v>
       </c>
       <c r="C22" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C23" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>23</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B27" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C27" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B28">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C28" s="1">
-        <v>900</v>
+        <f>Table3[[#This Row],[Units Contributed]]*60</f>
+        <v>780</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C29" s="1">
-        <v>540</v>
+        <f>Table3[[#This Row],[Units Contributed]]*60</f>
+        <v>480</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C30" s="1">
-        <v>360</v>
+        <f>Table3[[#This Row],[Units Contributed]]*60</f>
+        <v>300</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B31">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C31" s="1">
-        <v>480</v>
+        <f>Table3[[#This Row],[Units Contributed]]*60</f>
+        <v>300</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -932,19 +1195,20 @@
       </c>
       <c r="B32">
         <f>SUM(B28:B31)</f>
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="C32" s="1">
-        <f>SUM(C28:C31)</f>
-        <v>2280</v>
+        <f>Table3[[#This Row],[Units Contributed]]*60</f>
+        <v>1860</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
   <tableParts count="3">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>